<commit_message>
Format notes with markdown headings, fix normalization explanation, renumber files
</commit_message>
<xml_diff>
--- a/02_Image By Hand/02_CV C1 M1.xlsx
+++ b/02_Image By Hand/02_CV C1 M1.xlsx
@@ -1,51 +1,50 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29122"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://o365coloradoedu-my.sharepoint.com/personal/peye9704_colorado_edu/Documents/2025/Teach/CSCI5722-S25/Lectures/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1259" documentId="8_{E5D19860-1615-1C47-9036-2D40D7FFDBD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10FF4A88-821A-4815-91AD-934C63D995B7}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="17020" yWindow="1740" windowWidth="21800" windowHeight="26540" activeTab="1" xr2:uid="{3882FE0B-4295-864B-AC95-E6EA1D6CFBE9}"/>
+    <workbookView xWindow="17020" yWindow="1740" windowWidth="21800" windowHeight="26540" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="hand_blank" sheetId="1" r:id="rId1"/>
-    <sheet name="excel_blank" sheetId="2" r:id="rId2"/>
+    <sheet sheetId="1" name="hand_blank" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="excel_blank" state="visible" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191028"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="66">
   <si>
     <t>Image Array</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>7</t>
   </si>
   <si>
     <t>Image Matrix</t>
   </si>
   <si>
     <t>(width = 2)</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>(width = 3)</t>
@@ -57,7 +56,25 @@
     <t>(greater than 3)</t>
   </si>
   <si>
+    <t>0</t>
+  </si>
+  <si>
     <t>Byte Array</t>
+  </si>
+  <si>
+    <t>8 bits</t>
+  </si>
+  <si>
+    <t>255</t>
+  </si>
+  <si>
+    <t>128</t>
+  </si>
+  <si>
+    <t>42</t>
+  </si>
+  <si>
+    <t>30</t>
   </si>
   <si>
     <t>Range</t>
@@ -75,13 +92,46 @@
     <t>Double Array</t>
   </si>
   <si>
+    <t>0.5</t>
+  </si>
+  <si>
+    <t>-0.3</t>
+  </si>
+  <si>
+    <t>4305</t>
+  </si>
+  <si>
+    <t>-324</t>
+  </si>
+  <si>
+    <t>3.2</t>
+  </si>
+  <si>
     <t>Double Range</t>
+  </si>
+  <si>
+    <t>-3.4e+38</t>
+  </si>
+  <si>
+    <t>+3.4e+38</t>
   </si>
   <si>
     <t>Double Image Matrix</t>
   </si>
   <si>
     <t>Normalized Double Array</t>
+  </si>
+  <si>
+    <t>example</t>
+  </si>
+  <si>
+    <t>0.4</t>
+  </si>
+  <si>
+    <t>0.3</t>
+  </si>
+  <si>
+    <t>0.2</t>
   </si>
   <si>
     <t>RGB Values</t>
@@ -168,36 +218,43 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="0"/>
-      <name val="Aptos Narrow"/>
+      <color theme="1"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <color theme="0"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
     </font>
   </fonts>
   <fills count="10">
@@ -210,6 +267,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00FF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -246,12 +309,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF00FF"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00FF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -363,46 +420,36 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="11" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <mruColors>
-      <color rgb="FF0000FF"/>
-      <color rgb="FF00FF00"/>
-      <color rgb="FFFF0000"/>
-      <color rgb="FFFF00FF"/>
-      <color rgb="FF00FFFF"/>
-    </mruColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -730,497 +777,632 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FA66F01-CAB9-2447-A14E-1E86D3E83292}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L86"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
+  <sheetFormatPr defaultRowHeight="15.95" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="11" customHeight="1"/>
   <cols>
     <col min="1" max="38" width="4.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>1</v>
       </c>
+      <c r="B6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="C11" s="2" t="s">
+        <v>3</v>
+      </c>
     </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="7" spans="1:6">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
-    <row r="8" spans="1:6">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="10" spans="1:6">
-      <c r="A10" t="s">
-        <v>3</v>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="2"/>
     </row>
-    <row r="12" spans="1:6">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="14" spans="1:6">
-      <c r="A14" s="1" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>21</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>22</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>25</v>
+      </c>
+      <c r="B40" t="s">
+        <v>26</v>
+      </c>
+      <c r="C40" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="2"/>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B44" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E45" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="F45" s="2" t="s">
+        <v>37</v>
+      </c>
     </row>
-    <row r="15" spans="1:6">
-      <c r="A15" t="s">
-        <v>5</v>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" s="1" t="s">
+        <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>21</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="17" spans="1:6">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>22</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="19" spans="1:6">
-      <c r="A19" s="1" t="s">
-        <v>6</v>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" s="1" t="s">
+        <v>39</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
+    <row r="52" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B52" t="s">
+        <v>40</v>
+      </c>
+      <c r="F52" t="s">
+        <v>41</v>
+      </c>
     </row>
-    <row r="22" spans="1:6">
-      <c r="A22" s="1" t="s">
-        <v>7</v>
+    <row r="53" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B53" t="s">
+        <v>42</v>
+      </c>
+      <c r="C53" t="s">
+        <v>43</v>
+      </c>
+      <c r="D53" t="s">
+        <v>44</v>
+      </c>
+      <c r="F53" t="s">
+        <v>42</v>
+      </c>
+      <c r="G53" t="s">
+        <v>43</v>
+      </c>
+      <c r="H53" t="s">
+        <v>44</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
-      <c r="A23" t="s">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B54" s="2"/>
+      <c r="C54" s="2"/>
+      <c r="D54" s="2"/>
+      <c r="F54" s="2"/>
+      <c r="G54" s="2"/>
+      <c r="H54" s="2"/>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B55" s="2"/>
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+      <c r="F55" s="2"/>
+      <c r="G55" s="2"/>
+      <c r="H55" s="2"/>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B56" s="2"/>
+      <c r="C56" s="2"/>
+      <c r="D56" s="2"/>
+      <c r="F56" s="2"/>
+      <c r="G56" s="2"/>
+      <c r="H56" s="2"/>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B57" s="2"/>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="2"/>
+      <c r="H57" s="2"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B58" s="2"/>
+      <c r="C58" s="2"/>
+      <c r="D58" s="2"/>
+      <c r="F58" s="2"/>
+      <c r="G58" s="2"/>
+      <c r="H58" s="2"/>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="61" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B61" t="s">
+        <v>42</v>
+      </c>
+      <c r="C61" t="s">
+        <v>43</v>
+      </c>
+      <c r="D61" t="s">
+        <v>44</v>
+      </c>
+      <c r="F61" t="s">
+        <v>42</v>
+      </c>
+      <c r="G61" t="s">
+        <v>43</v>
+      </c>
+      <c r="H61" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A62" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B62" s="2"/>
+      <c r="C62" s="2"/>
+      <c r="D62" s="2"/>
+      <c r="F62" s="2"/>
+      <c r="G62" s="2"/>
+      <c r="H62" s="2"/>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A63" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B63" s="2"/>
+      <c r="C63" s="2"/>
+      <c r="D63" s="2"/>
+      <c r="F63" s="2"/>
+      <c r="G63" s="2"/>
+      <c r="H63" s="2"/>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A64" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="B64" s="2"/>
+      <c r="C64" s="2"/>
+      <c r="D64" s="2"/>
+      <c r="F64" s="2"/>
+      <c r="G64" s="2"/>
+      <c r="H64" s="2"/>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A67" s="2"/>
+      <c r="B67" s="2"/>
+      <c r="C67" s="2"/>
+      <c r="D67" s="2"/>
+      <c r="E67" s="2"/>
+      <c r="F67" s="2"/>
+      <c r="G67" s="2"/>
+      <c r="H67" s="2"/>
+      <c r="I67" s="2"/>
+      <c r="J67" s="2"/>
+      <c r="K67" s="2"/>
+      <c r="L67" s="2"/>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>45</v>
+      </c>
+      <c r="D69" t="s">
+        <v>51</v>
+      </c>
+      <c r="G69" t="s">
+        <v>52</v>
+      </c>
+      <c r="J69" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="3"/>
     </row>
-    <row r="24" spans="1:6">
-      <c r="A24" t="s">
-        <v>9</v>
-      </c>
-      <c r="B24" s="3"/>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" s="2"/>
+      <c r="B74" s="2"/>
     </row>
-    <row r="26" spans="1:6">
-      <c r="A26" s="1" t="s">
-        <v>10</v>
-      </c>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" s="2"/>
+      <c r="B75" s="12"/>
     </row>
-    <row r="27" spans="1:6">
-      <c r="A27" t="s">
-        <v>3</v>
-      </c>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" s="7"/>
     </row>
-    <row r="28" spans="1:6">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" s="1" t="s">
+        <v>56</v>
+      </c>
     </row>
-    <row r="29" spans="1:6">
-      <c r="A29" s="3"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B79" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="C79" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D79" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="E79" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="F79" s="15" t="s">
+        <v>59</v>
+      </c>
     </row>
-    <row r="31" spans="1:6">
-      <c r="A31" s="1" t="s">
-        <v>11</v>
-      </c>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" s="16"/>
+      <c r="C80" s="17"/>
+      <c r="D80" s="16"/>
+      <c r="F80" s="17"/>
     </row>
-    <row r="32" spans="1:6">
-      <c r="A32" s="3"/>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" s="16"/>
+      <c r="C81" s="17"/>
+      <c r="D81" s="16"/>
+      <c r="F81" s="17"/>
     </row>
-    <row r="34" spans="1:6">
-      <c r="A34" s="1" t="s">
-        <v>12</v>
-      </c>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" s="18"/>
+      <c r="B82" s="19"/>
+      <c r="C82" s="20"/>
+      <c r="D82" s="18"/>
+      <c r="E82" s="19"/>
+      <c r="F82" s="20"/>
     </row>
-    <row r="35" spans="1:6">
-      <c r="A35" t="s">
-        <v>8</v>
-      </c>
-      <c r="B35" s="19"/>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B83" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="C83" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D83" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="E83" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="F83" s="15" t="s">
+        <v>59</v>
+      </c>
     </row>
-    <row r="36" spans="1:6">
-      <c r="A36" t="s">
-        <v>9</v>
-      </c>
-      <c r="B36" s="20"/>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" s="16"/>
+      <c r="C84" s="17"/>
+      <c r="D84" s="16"/>
+      <c r="F84" s="17"/>
     </row>
-    <row r="38" spans="1:6">
-      <c r="A38" s="1" t="s">
-        <v>13</v>
-      </c>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" s="16"/>
+      <c r="C85" s="17"/>
+      <c r="D85" s="16"/>
+      <c r="F85" s="17"/>
     </row>
-    <row r="39" spans="1:6">
-      <c r="A39" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6">
-      <c r="A41" s="3"/>
-      <c r="B41" s="3"/>
-      <c r="C41" s="3"/>
-    </row>
-    <row r="42" spans="1:6">
-      <c r="A42" s="3"/>
-      <c r="B42" s="3"/>
-      <c r="C42" s="3"/>
-    </row>
-    <row r="44" spans="1:6">
-      <c r="A44" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6">
-      <c r="A45" s="3"/>
-      <c r="B45" s="3"/>
-      <c r="C45" s="3"/>
-      <c r="D45" s="3"/>
-      <c r="E45" s="3"/>
-      <c r="F45" s="3"/>
-    </row>
-    <row r="47" spans="1:6">
-      <c r="A47" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6">
-      <c r="A48" t="s">
-        <v>8</v>
-      </c>
-      <c r="B48" s="3"/>
-    </row>
-    <row r="49" spans="1:8">
-      <c r="A49" t="s">
-        <v>9</v>
-      </c>
-      <c r="B49" s="3"/>
-    </row>
-    <row r="51" spans="1:8">
-      <c r="A51" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8">
-      <c r="B52" t="s">
-        <v>16</v>
-      </c>
-      <c r="F52" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8">
-      <c r="B53" t="s">
-        <v>18</v>
-      </c>
-      <c r="C53" t="s">
-        <v>19</v>
-      </c>
-      <c r="D53" t="s">
-        <v>20</v>
-      </c>
-      <c r="F53" t="s">
-        <v>18</v>
-      </c>
-      <c r="G53" t="s">
-        <v>19</v>
-      </c>
-      <c r="H53" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8">
-      <c r="A54" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B54" s="3"/>
-      <c r="C54" s="3"/>
-      <c r="D54" s="3"/>
-      <c r="F54" s="3"/>
-      <c r="G54" s="3"/>
-      <c r="H54" s="3"/>
-    </row>
-    <row r="55" spans="1:8">
-      <c r="A55" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B55" s="3"/>
-      <c r="C55" s="3"/>
-      <c r="D55" s="3"/>
-      <c r="F55" s="3"/>
-      <c r="G55" s="3"/>
-      <c r="H55" s="3"/>
-    </row>
-    <row r="56" spans="1:8">
-      <c r="A56" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="B56" s="3"/>
-      <c r="C56" s="3"/>
-      <c r="D56" s="3"/>
-      <c r="F56" s="3"/>
-      <c r="G56" s="3"/>
-      <c r="H56" s="3"/>
-    </row>
-    <row r="57" spans="1:8">
-      <c r="A57" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B57" s="3"/>
-      <c r="C57" s="3"/>
-      <c r="D57" s="3"/>
-      <c r="F57" s="3"/>
-      <c r="G57" s="3"/>
-      <c r="H57" s="3"/>
-    </row>
-    <row r="58" spans="1:8">
-      <c r="A58" s="17" t="s">
-        <v>25</v>
-      </c>
-      <c r="B58" s="3"/>
-      <c r="C58" s="3"/>
-      <c r="D58" s="3"/>
-      <c r="F58" s="3"/>
-      <c r="G58" s="3"/>
-      <c r="H58" s="3"/>
-    </row>
-    <row r="60" spans="1:8">
-      <c r="A60" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="61" spans="1:8">
-      <c r="B61" t="s">
-        <v>18</v>
-      </c>
-      <c r="C61" t="s">
-        <v>19</v>
-      </c>
-      <c r="D61" t="s">
-        <v>20</v>
-      </c>
-      <c r="F61" t="s">
-        <v>18</v>
-      </c>
-      <c r="G61" t="s">
-        <v>19</v>
-      </c>
-      <c r="H61" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="62" spans="1:8">
-      <c r="A62" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B62" s="3"/>
-      <c r="C62" s="3"/>
-      <c r="D62" s="3"/>
-      <c r="F62" s="3"/>
-      <c r="G62" s="3"/>
-      <c r="H62" s="3"/>
-    </row>
-    <row r="63" spans="1:8">
-      <c r="A63" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B63" s="3"/>
-      <c r="C63" s="3"/>
-      <c r="D63" s="3"/>
-      <c r="F63" s="3"/>
-      <c r="G63" s="3"/>
-      <c r="H63" s="3"/>
-    </row>
-    <row r="64" spans="1:8">
-      <c r="A64" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B64" s="3"/>
-      <c r="C64" s="3"/>
-      <c r="D64" s="3"/>
-      <c r="F64" s="3"/>
-      <c r="G64" s="3"/>
-      <c r="H64" s="3"/>
-    </row>
-    <row r="66" spans="1:12">
-      <c r="A66" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="67" spans="1:12">
-      <c r="A67" s="3"/>
-      <c r="B67" s="3"/>
-      <c r="C67" s="3"/>
-      <c r="D67" s="3"/>
-      <c r="E67" s="3"/>
-      <c r="F67" s="3"/>
-      <c r="G67" s="3"/>
-      <c r="H67" s="3"/>
-      <c r="I67" s="3"/>
-      <c r="J67" s="3"/>
-      <c r="K67" s="3"/>
-      <c r="L67" s="3"/>
-    </row>
-    <row r="69" spans="1:12">
-      <c r="A69" t="s">
-        <v>21</v>
-      </c>
-      <c r="D69" t="s">
-        <v>27</v>
-      </c>
-      <c r="G69" t="s">
-        <v>28</v>
-      </c>
-      <c r="J69" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="72" spans="1:12">
-      <c r="A72" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="73" spans="1:12">
-      <c r="A73" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="74" spans="1:12">
-      <c r="A74" s="3"/>
-      <c r="B74" s="3"/>
-    </row>
-    <row r="75" spans="1:12">
-      <c r="A75" s="3"/>
-      <c r="B75" s="23"/>
-    </row>
-    <row r="76" spans="1:12">
-      <c r="A76" s="4"/>
-    </row>
-    <row r="77" spans="1:12">
-      <c r="A77" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="79" spans="1:12">
-      <c r="A79" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B79" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C79" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="D79" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="E79" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="F79" s="11" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="80" spans="1:12">
-      <c r="A80" s="12"/>
-      <c r="C80" s="13"/>
-      <c r="D80" s="12"/>
-      <c r="F80" s="13"/>
-    </row>
-    <row r="81" spans="1:6">
-      <c r="A81" s="12"/>
-      <c r="C81" s="13"/>
-      <c r="D81" s="12"/>
-      <c r="F81" s="13"/>
-    </row>
-    <row r="82" spans="1:6">
-      <c r="A82" s="14"/>
-      <c r="B82" s="15"/>
-      <c r="C82" s="16"/>
-      <c r="D82" s="14"/>
-      <c r="E82" s="15"/>
-      <c r="F82" s="16"/>
-    </row>
-    <row r="83" spans="1:6">
-      <c r="A83" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B83" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C83" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="D83" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="E83" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="F83" s="11" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6">
-      <c r="A84" s="12"/>
-      <c r="C84" s="13"/>
-      <c r="D84" s="12"/>
-      <c r="F84" s="13"/>
-    </row>
-    <row r="85" spans="1:6">
-      <c r="A85" s="12"/>
-      <c r="C85" s="13"/>
-      <c r="D85" s="12"/>
-      <c r="F85" s="13"/>
-    </row>
-    <row r="86" spans="1:6">
-      <c r="A86" s="14"/>
-      <c r="B86" s="15"/>
-      <c r="C86" s="16"/>
-      <c r="D86" s="14"/>
-      <c r="E86" s="15"/>
-      <c r="F86" s="16"/>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" s="18"/>
+      <c r="B86" s="19"/>
+      <c r="C86" s="20"/>
+      <c r="D86" s="18"/>
+      <c r="E86" s="19"/>
+      <c r="F86" s="20"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1228,21 +1410,21 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C8C5D22-8DD3-4194-AF64-20EF1BAB3E60}">
-  <dimension ref="A1:DND154"/>
-  <sheetFormatPr defaultColWidth="2.5" defaultRowHeight="15.95"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="F1:DND154"/>
+  <sheetFormatPr defaultRowHeight="15.95" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="2.5" customHeight="1"/>
   <cols>
-    <col min="1" max="9" width="2.625" bestFit="1" customWidth="1"/>
-    <col min="10" max="87" width="3.5" bestFit="1" customWidth="1"/>
-    <col min="88" max="96" width="2.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="9" width="2.625" customWidth="1"/>
+    <col min="10" max="87" width="3.5" customWidth="1"/>
+    <col min="88" max="96" width="2.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1024">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:1024">
+    <row r="2" spans="1:1024" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -4316,17 +4498,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1024">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
     </row>
-    <row r="5" spans="1:1024">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:1024">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A6" s="21"/>
       <c r="B6" s="21"/>
       <c r="C6" s="21"/>
@@ -4360,7 +4542,7 @@
       <c r="AE6" s="21"/>
       <c r="AF6" s="21"/>
     </row>
-    <row r="7" spans="1:1024">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A7" s="21"/>
       <c r="B7" s="21"/>
       <c r="C7" s="21"/>
@@ -4394,7 +4576,7 @@
       <c r="AE7" s="21"/>
       <c r="AF7" s="21"/>
     </row>
-    <row r="8" spans="1:1024">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A8" s="21"/>
       <c r="B8" s="21"/>
       <c r="C8" s="21"/>
@@ -4428,7 +4610,7 @@
       <c r="AE8" s="21"/>
       <c r="AF8" s="21"/>
     </row>
-    <row r="9" spans="1:1024">
+    <row r="9" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A9" s="21"/>
       <c r="B9" s="21"/>
       <c r="C9" s="21"/>
@@ -4462,7 +4644,7 @@
       <c r="AE9" s="21"/>
       <c r="AF9" s="21"/>
     </row>
-    <row r="10" spans="1:1024">
+    <row r="10" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A10" s="21"/>
       <c r="B10" s="21"/>
       <c r="C10" s="21"/>
@@ -4496,7 +4678,7 @@
       <c r="AE10" s="21"/>
       <c r="AF10" s="21"/>
     </row>
-    <row r="11" spans="1:1024">
+    <row r="11" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A11" s="21"/>
       <c r="B11" s="21"/>
       <c r="C11" s="21"/>
@@ -4530,7 +4712,7 @@
       <c r="AE11" s="21"/>
       <c r="AF11" s="21"/>
     </row>
-    <row r="12" spans="1:1024">
+    <row r="12" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A12" s="21"/>
       <c r="B12" s="21"/>
       <c r="C12" s="21"/>
@@ -4564,7 +4746,7 @@
       <c r="AE12" s="21"/>
       <c r="AF12" s="21"/>
     </row>
-    <row r="13" spans="1:1024">
+    <row r="13" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A13" s="21"/>
       <c r="B13" s="21"/>
       <c r="C13" s="21"/>
@@ -4598,7 +4780,7 @@
       <c r="AE13" s="21"/>
       <c r="AF13" s="21"/>
     </row>
-    <row r="14" spans="1:1024">
+    <row r="14" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A14" s="21"/>
       <c r="B14" s="21"/>
       <c r="C14" s="21"/>
@@ -4632,7 +4814,7 @@
       <c r="AE14" s="21"/>
       <c r="AF14" s="21"/>
     </row>
-    <row r="15" spans="1:1024">
+    <row r="15" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A15" s="21"/>
       <c r="B15" s="21"/>
       <c r="C15" s="21"/>
@@ -4666,7 +4848,7 @@
       <c r="AE15" s="21"/>
       <c r="AF15" s="21"/>
     </row>
-    <row r="16" spans="1:1024">
+    <row r="16" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A16" s="21"/>
       <c r="B16" s="21"/>
       <c r="C16" s="21"/>
@@ -4700,7 +4882,7 @@
       <c r="AE16" s="21"/>
       <c r="AF16" s="21"/>
     </row>
-    <row r="17" spans="1:32">
+    <row r="17" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A17" s="21"/>
       <c r="B17" s="21"/>
       <c r="C17" s="21"/>
@@ -4734,7 +4916,7 @@
       <c r="AE17" s="21"/>
       <c r="AF17" s="21"/>
     </row>
-    <row r="18" spans="1:32">
+    <row r="18" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A18" s="21"/>
       <c r="B18" s="21"/>
       <c r="C18" s="21"/>
@@ -4768,7 +4950,7 @@
       <c r="AE18" s="21"/>
       <c r="AF18" s="21"/>
     </row>
-    <row r="19" spans="1:32">
+    <row r="19" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A19" s="21"/>
       <c r="B19" s="21"/>
       <c r="C19" s="21"/>
@@ -4802,7 +4984,7 @@
       <c r="AE19" s="21"/>
       <c r="AF19" s="21"/>
     </row>
-    <row r="20" spans="1:32">
+    <row r="20" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A20" s="21"/>
       <c r="B20" s="21"/>
       <c r="C20" s="21"/>
@@ -4836,7 +5018,7 @@
       <c r="AE20" s="21"/>
       <c r="AF20" s="21"/>
     </row>
-    <row r="21" spans="1:32">
+    <row r="21" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A21" s="21"/>
       <c r="B21" s="21"/>
       <c r="C21" s="21"/>
@@ -4870,7 +5052,7 @@
       <c r="AE21" s="21"/>
       <c r="AF21" s="21"/>
     </row>
-    <row r="22" spans="1:32">
+    <row r="22" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A22" s="21"/>
       <c r="B22" s="21"/>
       <c r="C22" s="21"/>
@@ -4904,7 +5086,7 @@
       <c r="AE22" s="21"/>
       <c r="AF22" s="21"/>
     </row>
-    <row r="23" spans="1:32">
+    <row r="23" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A23" s="21"/>
       <c r="B23" s="21"/>
       <c r="C23" s="21"/>
@@ -4938,7 +5120,7 @@
       <c r="AE23" s="21"/>
       <c r="AF23" s="21"/>
     </row>
-    <row r="24" spans="1:32">
+    <row r="24" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A24" s="21"/>
       <c r="B24" s="21"/>
       <c r="C24" s="21"/>
@@ -4972,7 +5154,7 @@
       <c r="AE24" s="21"/>
       <c r="AF24" s="21"/>
     </row>
-    <row r="25" spans="1:32">
+    <row r="25" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A25" s="21"/>
       <c r="B25" s="21"/>
       <c r="C25" s="21"/>
@@ -5006,7 +5188,7 @@
       <c r="AE25" s="21"/>
       <c r="AF25" s="21"/>
     </row>
-    <row r="26" spans="1:32">
+    <row r="26" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A26" s="21"/>
       <c r="B26" s="21"/>
       <c r="C26" s="21"/>
@@ -5040,7 +5222,7 @@
       <c r="AE26" s="21"/>
       <c r="AF26" s="21"/>
     </row>
-    <row r="27" spans="1:32">
+    <row r="27" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A27" s="21"/>
       <c r="B27" s="21"/>
       <c r="C27" s="21"/>
@@ -5074,7 +5256,7 @@
       <c r="AE27" s="21"/>
       <c r="AF27" s="21"/>
     </row>
-    <row r="28" spans="1:32">
+    <row r="28" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A28" s="21"/>
       <c r="B28" s="21"/>
       <c r="C28" s="21"/>
@@ -5108,7 +5290,7 @@
       <c r="AE28" s="21"/>
       <c r="AF28" s="21"/>
     </row>
-    <row r="29" spans="1:32">
+    <row r="29" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A29" s="21"/>
       <c r="B29" s="21"/>
       <c r="C29" s="21"/>
@@ -5142,7 +5324,7 @@
       <c r="AE29" s="21"/>
       <c r="AF29" s="21"/>
     </row>
-    <row r="30" spans="1:32">
+    <row r="30" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A30" s="21"/>
       <c r="B30" s="21"/>
       <c r="C30" s="21"/>
@@ -5176,7 +5358,7 @@
       <c r="AE30" s="21"/>
       <c r="AF30" s="21"/>
     </row>
-    <row r="31" spans="1:32">
+    <row r="31" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A31" s="21"/>
       <c r="B31" s="21"/>
       <c r="C31" s="21"/>
@@ -5210,7 +5392,7 @@
       <c r="AE31" s="21"/>
       <c r="AF31" s="21"/>
     </row>
-    <row r="32" spans="1:32">
+    <row r="32" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A32" s="21"/>
       <c r="B32" s="21"/>
       <c r="C32" s="21"/>
@@ -5244,7 +5426,7 @@
       <c r="AE32" s="21"/>
       <c r="AF32" s="21"/>
     </row>
-    <row r="33" spans="1:32">
+    <row r="33" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A33" s="21"/>
       <c r="B33" s="21"/>
       <c r="C33" s="21"/>
@@ -5278,7 +5460,7 @@
       <c r="AE33" s="21"/>
       <c r="AF33" s="21"/>
     </row>
-    <row r="34" spans="1:32">
+    <row r="34" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A34" s="21"/>
       <c r="B34" s="21"/>
       <c r="C34" s="21"/>
@@ -5312,7 +5494,7 @@
       <c r="AE34" s="21"/>
       <c r="AF34" s="21"/>
     </row>
-    <row r="35" spans="1:32">
+    <row r="35" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A35" s="21"/>
       <c r="B35" s="21"/>
       <c r="C35" s="21"/>
@@ -5346,7 +5528,7 @@
       <c r="AE35" s="21"/>
       <c r="AF35" s="21"/>
     </row>
-    <row r="36" spans="1:32">
+    <row r="36" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A36" s="21"/>
       <c r="B36" s="21"/>
       <c r="C36" s="21"/>
@@ -5380,7 +5562,7 @@
       <c r="AE36" s="21"/>
       <c r="AF36" s="21"/>
     </row>
-    <row r="37" spans="1:32">
+    <row r="37" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A37" s="21"/>
       <c r="B37" s="21"/>
       <c r="C37" s="21"/>
@@ -5414,12 +5596,12 @@
       <c r="AE37" s="21"/>
       <c r="AF37" s="21"/>
     </row>
-    <row r="39" spans="1:32">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>38</v>
+        <v>62</v>
       </c>
     </row>
-    <row r="40" spans="1:32">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="22">
         <v>0</v>
       </c>
@@ -5436,7 +5618,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="42" spans="1:32">
+    <row r="42" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A42" s="22"/>
       <c r="B42" s="22"/>
       <c r="C42" s="22"/>
@@ -5470,7 +5652,7 @@
       <c r="AE42" s="22"/>
       <c r="AF42" s="22"/>
     </row>
-    <row r="43" spans="1:32">
+    <row r="43" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A43" s="22"/>
       <c r="B43" s="22"/>
       <c r="C43" s="22"/>
@@ -5504,7 +5686,7 @@
       <c r="AE43" s="22"/>
       <c r="AF43" s="22"/>
     </row>
-    <row r="44" spans="1:32">
+    <row r="44" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A44" s="22"/>
       <c r="B44" s="22"/>
       <c r="C44" s="22"/>
@@ -5538,7 +5720,7 @@
       <c r="AE44" s="22"/>
       <c r="AF44" s="22"/>
     </row>
-    <row r="45" spans="1:32">
+    <row r="45" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A45" s="22"/>
       <c r="B45" s="22"/>
       <c r="C45" s="22"/>
@@ -5572,7 +5754,7 @@
       <c r="AE45" s="22"/>
       <c r="AF45" s="22"/>
     </row>
-    <row r="46" spans="1:32">
+    <row r="46" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A46" s="22"/>
       <c r="B46" s="22"/>
       <c r="C46" s="22"/>
@@ -5606,7 +5788,7 @@
       <c r="AE46" s="22"/>
       <c r="AF46" s="22"/>
     </row>
-    <row r="47" spans="1:32">
+    <row r="47" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A47" s="22"/>
       <c r="B47" s="22"/>
       <c r="C47" s="22"/>
@@ -5640,7 +5822,7 @@
       <c r="AE47" s="22"/>
       <c r="AF47" s="22"/>
     </row>
-    <row r="48" spans="1:32">
+    <row r="48" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A48" s="22"/>
       <c r="B48" s="22"/>
       <c r="C48" s="22"/>
@@ -5674,7 +5856,7 @@
       <c r="AE48" s="22"/>
       <c r="AF48" s="22"/>
     </row>
-    <row r="49" spans="1:32">
+    <row r="49" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A49" s="22"/>
       <c r="B49" s="22"/>
       <c r="C49" s="22"/>
@@ -5708,7 +5890,7 @@
       <c r="AE49" s="22"/>
       <c r="AF49" s="22"/>
     </row>
-    <row r="50" spans="1:32">
+    <row r="50" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A50" s="22"/>
       <c r="B50" s="22"/>
       <c r="C50" s="22"/>
@@ -5742,7 +5924,7 @@
       <c r="AE50" s="22"/>
       <c r="AF50" s="22"/>
     </row>
-    <row r="51" spans="1:32">
+    <row r="51" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A51" s="22"/>
       <c r="B51" s="22"/>
       <c r="C51" s="22"/>
@@ -5776,7 +5958,7 @@
       <c r="AE51" s="22"/>
       <c r="AF51" s="22"/>
     </row>
-    <row r="52" spans="1:32">
+    <row r="52" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A52" s="22"/>
       <c r="B52" s="22"/>
       <c r="C52" s="22"/>
@@ -5810,7 +5992,7 @@
       <c r="AE52" s="22"/>
       <c r="AF52" s="22"/>
     </row>
-    <row r="53" spans="1:32">
+    <row r="53" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A53" s="22"/>
       <c r="B53" s="22"/>
       <c r="C53" s="22"/>
@@ -5844,7 +6026,7 @@
       <c r="AE53" s="22"/>
       <c r="AF53" s="22"/>
     </row>
-    <row r="54" spans="1:32">
+    <row r="54" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A54" s="22"/>
       <c r="B54" s="22"/>
       <c r="C54" s="22"/>
@@ -5878,7 +6060,7 @@
       <c r="AE54" s="22"/>
       <c r="AF54" s="22"/>
     </row>
-    <row r="55" spans="1:32">
+    <row r="55" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A55" s="22"/>
       <c r="B55" s="22"/>
       <c r="C55" s="22"/>
@@ -5912,7 +6094,7 @@
       <c r="AE55" s="22"/>
       <c r="AF55" s="22"/>
     </row>
-    <row r="56" spans="1:32">
+    <row r="56" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A56" s="22"/>
       <c r="B56" s="22"/>
       <c r="C56" s="22"/>
@@ -5946,7 +6128,7 @@
       <c r="AE56" s="22"/>
       <c r="AF56" s="22"/>
     </row>
-    <row r="57" spans="1:32">
+    <row r="57" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A57" s="22"/>
       <c r="B57" s="22"/>
       <c r="C57" s="22"/>
@@ -5980,7 +6162,7 @@
       <c r="AE57" s="22"/>
       <c r="AF57" s="22"/>
     </row>
-    <row r="58" spans="1:32">
+    <row r="58" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A58" s="22"/>
       <c r="B58" s="22"/>
       <c r="C58" s="22"/>
@@ -6014,7 +6196,7 @@
       <c r="AE58" s="22"/>
       <c r="AF58" s="22"/>
     </row>
-    <row r="59" spans="1:32">
+    <row r="59" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A59" s="22"/>
       <c r="B59" s="22"/>
       <c r="C59" s="22"/>
@@ -6048,7 +6230,7 @@
       <c r="AE59" s="22"/>
       <c r="AF59" s="22"/>
     </row>
-    <row r="60" spans="1:32">
+    <row r="60" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A60" s="22"/>
       <c r="B60" s="22"/>
       <c r="C60" s="22"/>
@@ -6082,7 +6264,7 @@
       <c r="AE60" s="22"/>
       <c r="AF60" s="22"/>
     </row>
-    <row r="61" spans="1:32">
+    <row r="61" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A61" s="22"/>
       <c r="B61" s="22"/>
       <c r="C61" s="22"/>
@@ -6116,7 +6298,7 @@
       <c r="AE61" s="22"/>
       <c r="AF61" s="22"/>
     </row>
-    <row r="62" spans="1:32">
+    <row r="62" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A62" s="22"/>
       <c r="B62" s="22"/>
       <c r="C62" s="22"/>
@@ -6150,7 +6332,7 @@
       <c r="AE62" s="22"/>
       <c r="AF62" s="22"/>
     </row>
-    <row r="63" spans="1:32">
+    <row r="63" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A63" s="22"/>
       <c r="B63" s="22"/>
       <c r="C63" s="22"/>
@@ -6184,7 +6366,7 @@
       <c r="AE63" s="22"/>
       <c r="AF63" s="22"/>
     </row>
-    <row r="64" spans="1:32">
+    <row r="64" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A64" s="22"/>
       <c r="B64" s="22"/>
       <c r="C64" s="22"/>
@@ -6218,7 +6400,7 @@
       <c r="AE64" s="22"/>
       <c r="AF64" s="22"/>
     </row>
-    <row r="65" spans="1:3072">
+    <row r="65" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A65" s="22"/>
       <c r="B65" s="22"/>
       <c r="C65" s="22"/>
@@ -6252,7 +6434,7 @@
       <c r="AE65" s="22"/>
       <c r="AF65" s="22"/>
     </row>
-    <row r="66" spans="1:3072">
+    <row r="66" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A66" s="22"/>
       <c r="B66" s="22"/>
       <c r="C66" s="22"/>
@@ -6286,7 +6468,7 @@
       <c r="AE66" s="22"/>
       <c r="AF66" s="22"/>
     </row>
-    <row r="67" spans="1:3072">
+    <row r="67" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A67" s="22"/>
       <c r="B67" s="22"/>
       <c r="C67" s="22"/>
@@ -6320,7 +6502,7 @@
       <c r="AE67" s="22"/>
       <c r="AF67" s="22"/>
     </row>
-    <row r="68" spans="1:3072">
+    <row r="68" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A68" s="22"/>
       <c r="B68" s="22"/>
       <c r="C68" s="22"/>
@@ -6354,7 +6536,7 @@
       <c r="AE68" s="22"/>
       <c r="AF68" s="22"/>
     </row>
-    <row r="69" spans="1:3072">
+    <row r="69" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A69" s="22"/>
       <c r="B69" s="22"/>
       <c r="C69" s="22"/>
@@ -6388,7 +6570,7 @@
       <c r="AE69" s="22"/>
       <c r="AF69" s="22"/>
     </row>
-    <row r="70" spans="1:3072">
+    <row r="70" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A70" s="22"/>
       <c r="B70" s="22"/>
       <c r="C70" s="22"/>
@@ -6422,7 +6604,7 @@
       <c r="AE70" s="22"/>
       <c r="AF70" s="22"/>
     </row>
-    <row r="71" spans="1:3072">
+    <row r="71" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A71" s="22"/>
       <c r="B71" s="22"/>
       <c r="C71" s="22"/>
@@ -6456,7 +6638,7 @@
       <c r="AE71" s="22"/>
       <c r="AF71" s="22"/>
     </row>
-    <row r="72" spans="1:3072">
+    <row r="72" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A72" s="22"/>
       <c r="B72" s="22"/>
       <c r="C72" s="22"/>
@@ -6490,7 +6672,7 @@
       <c r="AE72" s="22"/>
       <c r="AF72" s="22"/>
     </row>
-    <row r="73" spans="1:3072">
+    <row r="73" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A73" s="22"/>
       <c r="B73" s="22"/>
       <c r="C73" s="22"/>
@@ -6524,12 +6706,12 @@
       <c r="AE73" s="22"/>
       <c r="AF73" s="22"/>
     </row>
-    <row r="76" spans="1:3072">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
     </row>
-    <row r="77" spans="1:3072">
+    <row r="77" spans="1:3072" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>0</v>
       </c>
@@ -15747,17 +15929,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:3072">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
-        <v>39</v>
+        <v>63</v>
       </c>
     </row>
-    <row r="114" spans="1:9">
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
-        <v>40</v>
+        <v>64</v>
       </c>
     </row>
-    <row r="115" spans="1:9" ht="60" customHeight="1">
+    <row r="115" ht="60" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115" s="21">
         <v>255</v>
       </c>
@@ -15786,44 +15968,44 @@
         <v>255</v>
       </c>
     </row>
-    <row r="118" spans="1:9">
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
-        <v>41</v>
+        <v>65</v>
       </c>
     </row>
-    <row r="119" spans="1:9" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="120" spans="1:9" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="121" spans="1:9" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="122" spans="1:9" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="123" spans="1:9" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="124" spans="1:9" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="125" spans="1:9" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="126" spans="1:9" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="127" spans="1:9" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="128" spans="1:9" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="129" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="130" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="131" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="132" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="133" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="134" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="135" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="136" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="137" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="138" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="139" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="140" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="141" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="142" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="143" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="144" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="145" spans="6:6" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="146" spans="6:6" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="147" spans="6:6" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="148" spans="6:6" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="149" spans="6:6" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="150" spans="6:6" s="21" customFormat="1" ht="60" customHeight="1"/>
-    <row r="154" spans="6:6">
+    <row r="119" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="120" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="121" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="122" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="123" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="124" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="125" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="126" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="127" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="128" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="129" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="130" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="131" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="132" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="133" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="134" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="135" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="136" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="137" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="138" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="139" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="140" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="141" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="142" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="143" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="144" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="145" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="146" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="147" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="148" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="149" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="150" ht="60" customHeight="1" s="21" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="154" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F154" s="22"/>
     </row>
   </sheetData>
@@ -15949,378 +16131,4 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="9f339653-0c01-4318-ae97-7b543795deb4" xsi:nil="true"/>
-    <LikesCount xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Instructor xmlns="808fd839-170a-44a4-85e4-5aff044f8a2d" xsi:nil="true"/>
-    <Ratings xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="808fd839-170a-44a4-85e4-5aff044f8a2d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <LikedBy xmlns="http://schemas.microsoft.com/sharepoint/v3">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </LikedBy>
-    <Program_x0020_Affiliation xmlns="808fd839-170a-44a4-85e4-5aff044f8a2d">MS-EE</Program_x0020_Affiliation>
-    <RatedBy xmlns="http://schemas.microsoft.com/sharepoint/v3">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </RatedBy>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010055D1C97D5F27A942A6ECCDFB95DF13FE" ma:contentTypeVersion="26" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9e6a3a7b4fb9f8f917417f476f40303e">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="808fd839-170a-44a4-85e4-5aff044f8a2d" xmlns:ns3="9f339653-0c01-4318-ae97-7b543795deb4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="870ad7e9e8b8d606b6943cd501d3d7d1" ns1:_="" ns2:_="" ns3:_="">
-    <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
-    <xsd:import namespace="808fd839-170a-44a4-85e4-5aff044f8a2d"/>
-    <xsd:import namespace="9f339653-0c01-4318-ae97-7b543795deb4"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:Instructor" minOccurs="0"/>
-                <xsd:element ref="ns2:Program_x0020_Affiliation" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns1:AverageRating" minOccurs="0"/>
-                <xsd:element ref="ns1:RatingCount" minOccurs="0"/>
-                <xsd:element ref="ns1:RatedBy" minOccurs="0"/>
-                <xsd:element ref="ns1:Ratings" minOccurs="0"/>
-                <xsd:element ref="ns1:LikesCount" minOccurs="0"/>
-                <xsd:element ref="ns1:LikedBy" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="http://schemas.microsoft.com/sharepoint/v3" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="AverageRating" ma:index="25" nillable="true" ma:displayName="Rating (0-5)" ma:decimals="2" ma:description="Average value of all the ratings that have been submitted" ma:internalName="AverageRating" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Number"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="RatingCount" ma:index="26" nillable="true" ma:displayName="Number of Ratings" ma:decimals="0" ma:description="Number of ratings submitted" ma:internalName="RatingCount" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Number"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="RatedBy" ma:index="27" nillable="true" ma:displayName="Rated By" ma:description="Users rated the item." ma:hidden="true" ma:list="UserInfo" ma:internalName="RatedBy">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="Ratings" ma:index="28" nillable="true" ma:displayName="User ratings" ma:description="User ratings for the item" ma:hidden="true" ma:internalName="Ratings">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="LikesCount" ma:index="29" nillable="true" ma:displayName="Number of Likes" ma:internalName="LikesCount">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="LikedBy" ma:index="30" nillable="true" ma:displayName="Liked By" ma:hidden="true" ma:list="UserInfo" ma:internalName="LikedBy">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="808fd839-170a-44a4-85e4-5aff044f8a2d" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Instructor" ma:index="10" nillable="true" ma:displayName="Instructor" ma:format="Dropdown" ma:internalName="Instructor">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="Program_x0020_Affiliation" ma:index="11" nillable="true" ma:displayName="Program Affiliation" ma:default="MS-EE" ma:format="Dropdown" ma:internalName="Program_x0020_Affiliation">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Choice">
-          <xsd:enumeration value="MS-EE"/>
-          <xsd:enumeration value="MS-DS"/>
-          <xsd:enumeration value="ME-EM"/>
-          <xsd:enumeration value="Non-Credit"/>
-          <xsd:enumeration value="MS-CS"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="15" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="16" nillable="true" ma:displayName="Location" ma:description="" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="20" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="52802cc5-2881-4dd7-9d75-38905e9cf7fb" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="22" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="23" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:description="" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="24" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="9f339653-0c01-4318-ae97-7b543795deb4" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="12" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="13" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="TaxCatchAll" ma:index="21" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{7af0b387-c937-4d03-a801-ab4615f1d031}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="9f339653-0c01-4318-ae97-7b543795deb4">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1D4B1699-E1B9-41B2-8FE3-88CEB3CA849B}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1AAA3C0A-69F7-4337-A6D8-4FFEA56C4F9A}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51D9F78E-EFDC-4D7A-8F46-7AB1F250641E}"/>
 </file>
</xml_diff>